<commit_message>
added correlation analyses and reworked some graphs
</commit_message>
<xml_diff>
--- a/Results/01_UVC_CPD_percentage_pvals_dose.xlsx
+++ b/Results/01_UVC_CPD_percentage_pvals_dose.xlsx
@@ -1,115 +1,121 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr date1904="false"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Aktuell\Eigene Dateien\Eigene Dateien_Marc\R\Github\EKB\BFS_UVC\Results\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12030"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
-  <si>
-    <t xml:space="preserve">Location</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Origin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">.y.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">group1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">group2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">n1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">n2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">statistic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">p</t>
-  </si>
-  <si>
-    <t xml:space="preserve">p.adj</t>
-  </si>
-  <si>
-    <t xml:space="preserve">p.adj.signif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">effect</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Basal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">254nm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Old_skin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Count_perc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0 J/m²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30 J/m²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dose</t>
-  </si>
-  <si>
-    <t xml:space="preserve">300 J/m²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1000 J/m²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">***</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2000 J/m²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">**</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Young_skin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Suprabasal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">222nm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">*</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="30">
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Origin</t>
+  </si>
+  <si>
+    <t>.y.</t>
+  </si>
+  <si>
+    <t>group1</t>
+  </si>
+  <si>
+    <t>group2</t>
+  </si>
+  <si>
+    <t>n1</t>
+  </si>
+  <si>
+    <t>n2</t>
+  </si>
+  <si>
+    <t>statistic</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>p.adj</t>
+  </si>
+  <si>
+    <t>p.adj.signif</t>
+  </si>
+  <si>
+    <t>effect</t>
+  </si>
+  <si>
+    <t>Basal</t>
+  </si>
+  <si>
+    <t>222nm</t>
+  </si>
+  <si>
+    <t>Old_skin</t>
+  </si>
+  <si>
+    <t>Count_perc</t>
+  </si>
+  <si>
+    <t>0 J/m²</t>
+  </si>
+  <si>
+    <t>30 J/m²</t>
+  </si>
+  <si>
+    <t>ns</t>
+  </si>
+  <si>
+    <t>Dose</t>
+  </si>
+  <si>
+    <t>300 J/m²</t>
+  </si>
+  <si>
+    <t>1000 J/m²</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>2000 J/m²</t>
+  </si>
+  <si>
+    <t>254nm</t>
+  </si>
+  <si>
+    <t>***</t>
+  </si>
+  <si>
+    <t>**</t>
+  </si>
+  <si>
+    <t>Young_skin</t>
+  </si>
+  <si>
+    <t>Suprabasal</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -142,9 +148,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -426,11 +441,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:M33"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -471,7 +486,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -490,20 +505,20 @@
       <c r="F2" t="s">
         <v>18</v>
       </c>
-      <c r="G2" t="n">
-        <v>11</v>
-      </c>
-      <c r="H2" t="n">
-        <v>11</v>
-      </c>
-      <c r="I2" t="n">
-        <v>35.5</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0.13859649122807</v>
+      <c r="G2">
+        <v>11</v>
+      </c>
+      <c r="H2">
+        <v>11</v>
+      </c>
+      <c r="I2">
+        <v>79.5</v>
+      </c>
+      <c r="J2">
+        <v>0.20799999999999999</v>
+      </c>
+      <c r="K2">
+        <v>0.30374603174603199</v>
       </c>
       <c r="L2" t="s">
         <v>19</v>
@@ -512,7 +527,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -531,20 +546,20 @@
       <c r="F3" t="s">
         <v>21</v>
       </c>
-      <c r="G3" t="n">
-        <v>11</v>
-      </c>
-      <c r="H3" t="n">
-        <v>11</v>
-      </c>
-      <c r="I3" t="n">
-        <v>41</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.202</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.261606557377049</v>
+      <c r="G3">
+        <v>11</v>
+      </c>
+      <c r="H3">
+        <v>11</v>
+      </c>
+      <c r="I3">
+        <v>88</v>
+      </c>
+      <c r="J3">
+        <v>6.5000000000000002E-2</v>
+      </c>
+      <c r="K3">
+        <v>0.11694615384615401</v>
       </c>
       <c r="L3" t="s">
         <v>19</v>
@@ -553,7 +568,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -572,20 +587,20 @@
       <c r="F4" t="s">
         <v>22</v>
       </c>
-      <c r="G4" t="n">
-        <v>11</v>
-      </c>
-      <c r="H4" t="n">
-        <v>11</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.0000627</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0.0004898</v>
+      <c r="G4">
+        <v>11</v>
+      </c>
+      <c r="H4">
+        <v>11</v>
+      </c>
+      <c r="I4">
+        <v>99</v>
+      </c>
+      <c r="J4">
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="K4">
+        <v>2.4352941176470601E-2</v>
       </c>
       <c r="L4" t="s">
         <v>23</v>
@@ -594,7 +609,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -613,37 +628,37 @@
       <c r="F5" t="s">
         <v>24</v>
       </c>
-      <c r="G5" t="n">
-        <v>11</v>
-      </c>
-      <c r="H5" t="n">
-        <v>11</v>
-      </c>
-      <c r="I5" t="n">
-        <v>11</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0.00232352941176471</v>
+      <c r="G5">
+        <v>11</v>
+      </c>
+      <c r="H5">
+        <v>11</v>
+      </c>
+      <c r="I5">
+        <v>68.5</v>
+      </c>
+      <c r="J5">
+        <v>0.61199999999999999</v>
+      </c>
+      <c r="K5">
+        <v>0.70379999999999998</v>
       </c>
       <c r="L5" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="M5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="B6" t="s">
         <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="D6" t="s">
         <v>16</v>
@@ -654,20 +669,20 @@
       <c r="F6" t="s">
         <v>18</v>
       </c>
-      <c r="G6" t="n">
-        <v>10</v>
-      </c>
-      <c r="H6" t="n">
-        <v>10</v>
-      </c>
-      <c r="I6" t="n">
-        <v>72</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0.087</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0.124963636363636</v>
+      <c r="G6">
+        <v>11</v>
+      </c>
+      <c r="H6">
+        <v>11</v>
+      </c>
+      <c r="I6">
+        <v>33.5</v>
+      </c>
+      <c r="J6">
+        <v>7.0999999999999994E-2</v>
+      </c>
+      <c r="K6">
+        <v>0.12096296296296299</v>
       </c>
       <c r="L6" t="s">
         <v>19</v>
@@ -676,15 +691,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="D7" t="s">
         <v>16</v>
@@ -695,20 +710,20 @@
       <c r="F7" t="s">
         <v>21</v>
       </c>
-      <c r="G7" t="n">
-        <v>10</v>
-      </c>
-      <c r="H7" t="n">
-        <v>10</v>
-      </c>
-      <c r="I7" t="n">
-        <v>52</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0.906</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0.95432</v>
+      <c r="G7">
+        <v>11</v>
+      </c>
+      <c r="H7">
+        <v>11</v>
+      </c>
+      <c r="I7">
+        <v>40.5</v>
+      </c>
+      <c r="J7">
+        <v>0.187</v>
+      </c>
+      <c r="K7">
+        <v>0.28203278688524602</v>
       </c>
       <c r="L7" t="s">
         <v>19</v>
@@ -717,15 +732,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="B8" t="s">
         <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="D8" t="s">
         <v>16</v>
@@ -736,37 +751,37 @@
       <c r="F8" t="s">
         <v>22</v>
       </c>
-      <c r="G8" t="n">
-        <v>10</v>
-      </c>
-      <c r="H8" t="n">
-        <v>10</v>
-      </c>
-      <c r="I8" t="n">
-        <v>30</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0.131</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0.178431034482759</v>
+      <c r="G8">
+        <v>11</v>
+      </c>
+      <c r="H8">
+        <v>11</v>
+      </c>
+      <c r="I8">
+        <v>20.5</v>
+      </c>
+      <c r="J8">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="K8">
+        <v>1.9515151515151499E-2</v>
       </c>
       <c r="L8" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="M8" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="B9" t="s">
         <v>14</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="D9" t="s">
         <v>16</v>
@@ -777,34 +792,34 @@
       <c r="F9" t="s">
         <v>24</v>
       </c>
-      <c r="G9" t="n">
-        <v>10</v>
-      </c>
-      <c r="H9" t="n">
-        <v>10</v>
-      </c>
-      <c r="I9" t="n">
-        <v>23.5</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0.042</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0.0650588235294118</v>
+      <c r="G9">
+        <v>11</v>
+      </c>
+      <c r="H9">
+        <v>11</v>
+      </c>
+      <c r="I9">
+        <v>13</v>
+      </c>
+      <c r="J9">
+        <v>2E-3</v>
+      </c>
+      <c r="K9">
+        <v>7.3600000000000002E-3</v>
       </c>
       <c r="L9" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="M9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C10" t="s">
         <v>15</v>
@@ -818,20 +833,20 @@
       <c r="F10" t="s">
         <v>18</v>
       </c>
-      <c r="G10" t="n">
-        <v>11</v>
-      </c>
-      <c r="H10" t="n">
-        <v>11</v>
-      </c>
-      <c r="I10" t="n">
-        <v>33.5</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0.071</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0.10387037037037</v>
+      <c r="G10">
+        <v>11</v>
+      </c>
+      <c r="H10">
+        <v>11</v>
+      </c>
+      <c r="I10">
+        <v>35.5</v>
+      </c>
+      <c r="J10">
+        <v>0.1</v>
+      </c>
+      <c r="K10">
+        <v>0.16428571428571401</v>
       </c>
       <c r="L10" t="s">
         <v>19</v>
@@ -840,12 +855,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C11" t="s">
         <v>15</v>
@@ -859,20 +874,20 @@
       <c r="F11" t="s">
         <v>21</v>
       </c>
-      <c r="G11" t="n">
-        <v>11</v>
-      </c>
-      <c r="H11" t="n">
-        <v>11</v>
-      </c>
-      <c r="I11" t="n">
-        <v>40.5</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0.187</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0.246216666666667</v>
+      <c r="G11">
+        <v>11</v>
+      </c>
+      <c r="H11">
+        <v>11</v>
+      </c>
+      <c r="I11">
+        <v>41</v>
+      </c>
+      <c r="J11">
+        <v>0.20200000000000001</v>
+      </c>
+      <c r="K11">
+        <v>0.29974193548387101</v>
       </c>
       <c r="L11" t="s">
         <v>19</v>
@@ -881,12 +896,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C12" t="s">
         <v>15</v>
@@ -900,34 +915,34 @@
       <c r="F12" t="s">
         <v>22</v>
       </c>
-      <c r="G12" t="n">
-        <v>11</v>
-      </c>
-      <c r="H12" t="n">
-        <v>11</v>
-      </c>
-      <c r="I12" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0.0120217391304348</v>
+      <c r="G12">
+        <v>11</v>
+      </c>
+      <c r="H12">
+        <v>11</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>6.2700000000000006E-5</v>
+      </c>
+      <c r="K12">
+        <v>7.4611999999999996E-4</v>
       </c>
       <c r="L12" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="M12" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C13" t="s">
         <v>15</v>
@@ -941,34 +956,34 @@
       <c r="F13" t="s">
         <v>24</v>
       </c>
-      <c r="G13" t="n">
-        <v>11</v>
-      </c>
-      <c r="H13" t="n">
-        <v>11</v>
-      </c>
-      <c r="I13" t="n">
-        <v>13</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0.00427027027027027</v>
+      <c r="G13">
+        <v>11</v>
+      </c>
+      <c r="H13">
+        <v>11</v>
+      </c>
+      <c r="I13">
+        <v>11</v>
+      </c>
+      <c r="J13">
+        <v>1E-3</v>
+      </c>
+      <c r="K13">
+        <v>4.1818181818181798E-3</v>
       </c>
       <c r="L13" t="s">
+        <v>27</v>
+      </c>
+      <c r="M13" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" t="s">
         <v>25</v>
-      </c>
-      <c r="M13" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" t="s">
-        <v>14</v>
       </c>
       <c r="C14" t="s">
         <v>15</v>
@@ -982,34 +997,34 @@
       <c r="F14" t="s">
         <v>18</v>
       </c>
-      <c r="G14" t="n">
-        <v>11</v>
-      </c>
-      <c r="H14" t="n">
-        <v>11</v>
-      </c>
-      <c r="I14" t="n">
+      <c r="G14">
+        <v>11</v>
+      </c>
+      <c r="H14">
+        <v>11</v>
+      </c>
+      <c r="I14">
         <v>0</v>
       </c>
-      <c r="J14" t="n">
-        <v>0.000059</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0.0004898</v>
+      <c r="J14">
+        <v>5.8999999999999998E-5</v>
+      </c>
+      <c r="K14">
+        <v>7.4611999999999996E-4</v>
       </c>
       <c r="L14" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="M14" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B15" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="C15" t="s">
         <v>15</v>
@@ -1023,34 +1038,34 @@
       <c r="F15" t="s">
         <v>21</v>
       </c>
-      <c r="G15" t="n">
-        <v>11</v>
-      </c>
-      <c r="H15" t="n">
-        <v>11</v>
-      </c>
-      <c r="I15" t="n">
+      <c r="G15">
+        <v>11</v>
+      </c>
+      <c r="H15">
+        <v>11</v>
+      </c>
+      <c r="I15">
         <v>0</v>
       </c>
-      <c r="J15" t="n">
-        <v>0.0000593</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0.0004898</v>
+      <c r="J15">
+        <v>5.9299999999999998E-5</v>
+      </c>
+      <c r="K15">
+        <v>7.4611999999999996E-4</v>
       </c>
       <c r="L15" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="M15" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B16" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="C16" t="s">
         <v>15</v>
@@ -1064,34 +1079,34 @@
       <c r="F16" t="s">
         <v>22</v>
       </c>
-      <c r="G16" t="n">
-        <v>11</v>
-      </c>
-      <c r="H16" t="n">
-        <v>11</v>
-      </c>
-      <c r="I16" t="n">
+      <c r="G16">
+        <v>11</v>
+      </c>
+      <c r="H16">
+        <v>11</v>
+      </c>
+      <c r="I16">
         <v>0</v>
       </c>
-      <c r="J16" t="n">
-        <v>0.0000593</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0.0004898</v>
+      <c r="J16">
+        <v>5.9299999999999998E-5</v>
+      </c>
+      <c r="K16">
+        <v>7.4611999999999996E-4</v>
       </c>
       <c r="L16" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="M16" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B17" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="C17" t="s">
         <v>15</v>
@@ -1105,37 +1120,37 @@
       <c r="F17" t="s">
         <v>24</v>
       </c>
-      <c r="G17" t="n">
-        <v>11</v>
-      </c>
-      <c r="H17" t="n">
-        <v>11</v>
-      </c>
-      <c r="I17" t="n">
+      <c r="G17">
+        <v>11</v>
+      </c>
+      <c r="H17">
+        <v>11</v>
+      </c>
+      <c r="I17">
         <v>0</v>
       </c>
-      <c r="J17" t="n">
-        <v>0.0000593</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0.0004898</v>
+      <c r="J17">
+        <v>5.9299999999999998E-5</v>
+      </c>
+      <c r="K17">
+        <v>7.4611999999999996E-4</v>
       </c>
       <c r="L17" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="M17" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="B18" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" t="s">
         <v>28</v>
-      </c>
-      <c r="C18" t="s">
-        <v>26</v>
       </c>
       <c r="D18" t="s">
         <v>16</v>
@@ -1146,20 +1161,20 @@
       <c r="F18" t="s">
         <v>18</v>
       </c>
-      <c r="G18" t="n">
-        <v>10</v>
-      </c>
-      <c r="H18" t="n">
-        <v>10</v>
-      </c>
-      <c r="I18" t="n">
-        <v>25</v>
-      </c>
-      <c r="J18" t="n">
-        <v>0.056</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0.0834716981132075</v>
+      <c r="G18">
+        <v>10</v>
+      </c>
+      <c r="H18">
+        <v>10</v>
+      </c>
+      <c r="I18">
+        <v>62</v>
+      </c>
+      <c r="J18">
+        <v>0.36299999999999999</v>
+      </c>
+      <c r="K18">
+        <v>0.46383333333333299</v>
       </c>
       <c r="L18" t="s">
         <v>19</v>
@@ -1168,15 +1183,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="B19" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" t="s">
         <v>28</v>
-      </c>
-      <c r="C19" t="s">
-        <v>26</v>
       </c>
       <c r="D19" t="s">
         <v>16</v>
@@ -1187,20 +1202,20 @@
       <c r="F19" t="s">
         <v>21</v>
       </c>
-      <c r="G19" t="n">
-        <v>10</v>
-      </c>
-      <c r="H19" t="n">
-        <v>10</v>
-      </c>
-      <c r="I19" t="n">
-        <v>25</v>
-      </c>
-      <c r="J19" t="n">
-        <v>0.056</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0.0834716981132075</v>
+      <c r="G19">
+        <v>10</v>
+      </c>
+      <c r="H19">
+        <v>10</v>
+      </c>
+      <c r="I19">
+        <v>77</v>
+      </c>
+      <c r="J19">
+        <v>3.5999999999999997E-2</v>
+      </c>
+      <c r="K19">
+        <v>6.9469387755102002E-2</v>
       </c>
       <c r="L19" t="s">
         <v>19</v>
@@ -1209,15 +1224,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="B20" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" t="s">
         <v>28</v>
-      </c>
-      <c r="C20" t="s">
-        <v>26</v>
       </c>
       <c r="D20" t="s">
         <v>16</v>
@@ -1228,20 +1243,20 @@
       <c r="F20" t="s">
         <v>22</v>
       </c>
-      <c r="G20" t="n">
-        <v>10</v>
-      </c>
-      <c r="H20" t="n">
-        <v>10</v>
-      </c>
-      <c r="I20" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="J20" t="n">
-        <v>0.000285</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0.000938125</v>
+      <c r="G20">
+        <v>10</v>
+      </c>
+      <c r="H20">
+        <v>10</v>
+      </c>
+      <c r="I20">
+        <v>80.5</v>
+      </c>
+      <c r="J20">
+        <v>1.7000000000000001E-2</v>
+      </c>
+      <c r="K20">
+        <v>3.9043902439024399E-2</v>
       </c>
       <c r="L20" t="s">
         <v>23</v>
@@ -1250,15 +1265,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="B21" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21" t="s">
         <v>28</v>
-      </c>
-      <c r="C21" t="s">
-        <v>26</v>
       </c>
       <c r="D21" t="s">
         <v>16</v>
@@ -1269,37 +1284,37 @@
       <c r="F21" t="s">
         <v>24</v>
       </c>
-      <c r="G21" t="n">
-        <v>10</v>
-      </c>
-      <c r="H21" t="n">
-        <v>10</v>
-      </c>
-      <c r="I21" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="J21" t="n">
-        <v>0.000283</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0.000938125</v>
+      <c r="G21">
+        <v>10</v>
+      </c>
+      <c r="H21">
+        <v>10</v>
+      </c>
+      <c r="I21">
+        <v>78.5</v>
+      </c>
+      <c r="J21">
+        <v>2.5999999999999999E-2</v>
+      </c>
+      <c r="K21">
+        <v>5.5627906976744197E-2</v>
       </c>
       <c r="L21" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="M21" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B22" t="s">
         <v>14</v>
       </c>
       <c r="C22" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D22" t="s">
         <v>16</v>
@@ -1310,37 +1325,37 @@
       <c r="F22" t="s">
         <v>18</v>
       </c>
-      <c r="G22" t="n">
-        <v>10</v>
-      </c>
-      <c r="H22" t="n">
-        <v>10</v>
-      </c>
-      <c r="I22" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0.000144</v>
-      </c>
-      <c r="K22" t="n">
-        <v>0.000602894736842105</v>
+      <c r="G22">
+        <v>10</v>
+      </c>
+      <c r="H22">
+        <v>10</v>
+      </c>
+      <c r="I22">
+        <v>22.5</v>
+      </c>
+      <c r="J22">
+        <v>3.6999999999999998E-2</v>
+      </c>
+      <c r="K22">
+        <v>6.9469387755102002E-2</v>
       </c>
       <c r="L22" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="M22" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B23" t="s">
         <v>14</v>
       </c>
       <c r="C23" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D23" t="s">
         <v>16</v>
@@ -1351,37 +1366,37 @@
       <c r="F23" t="s">
         <v>21</v>
       </c>
-      <c r="G23" t="n">
-        <v>10</v>
-      </c>
-      <c r="H23" t="n">
-        <v>10</v>
-      </c>
-      <c r="I23" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" t="n">
-        <v>0.000145</v>
-      </c>
-      <c r="K23" t="n">
-        <v>0.000602894736842105</v>
+      <c r="G23">
+        <v>10</v>
+      </c>
+      <c r="H23">
+        <v>10</v>
+      </c>
+      <c r="I23">
+        <v>22.5</v>
+      </c>
+      <c r="J23">
+        <v>3.6999999999999998E-2</v>
+      </c>
+      <c r="K23">
+        <v>6.9469387755102002E-2</v>
       </c>
       <c r="L23" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="M23" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B24" t="s">
         <v>14</v>
       </c>
       <c r="C24" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D24" t="s">
         <v>16</v>
@@ -1392,37 +1407,37 @@
       <c r="F24" t="s">
         <v>22</v>
       </c>
-      <c r="G24" t="n">
-        <v>10</v>
-      </c>
-      <c r="H24" t="n">
-        <v>10</v>
-      </c>
-      <c r="I24" t="n">
+      <c r="G24">
+        <v>10</v>
+      </c>
+      <c r="H24">
+        <v>10</v>
+      </c>
+      <c r="I24">
         <v>0</v>
       </c>
-      <c r="J24" t="n">
-        <v>0.000144</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0.000602894736842105</v>
+      <c r="J24">
+        <v>1.45E-4</v>
+      </c>
+      <c r="K24">
+        <v>8.8933333333333301E-4</v>
       </c>
       <c r="L24" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="M24" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B25" t="s">
         <v>14</v>
       </c>
       <c r="C25" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D25" t="s">
         <v>16</v>
@@ -1433,30 +1448,361 @@
       <c r="F25" t="s">
         <v>24</v>
       </c>
-      <c r="G25" t="n">
-        <v>10</v>
-      </c>
-      <c r="H25" t="n">
-        <v>10</v>
-      </c>
-      <c r="I25" t="n">
+      <c r="G25">
+        <v>10</v>
+      </c>
+      <c r="H25">
+        <v>10</v>
+      </c>
+      <c r="I25">
+        <v>2.5</v>
+      </c>
+      <c r="J25">
+        <v>2.8299999999999999E-4</v>
+      </c>
+      <c r="K25">
+        <v>1.3018000000000001E-3</v>
+      </c>
+      <c r="L25" t="s">
+        <v>27</v>
+      </c>
+      <c r="M25" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>13</v>
+      </c>
+      <c r="B26" t="s">
+        <v>25</v>
+      </c>
+      <c r="C26" t="s">
+        <v>28</v>
+      </c>
+      <c r="D26" t="s">
+        <v>16</v>
+      </c>
+      <c r="E26" t="s">
+        <v>17</v>
+      </c>
+      <c r="F26" t="s">
+        <v>18</v>
+      </c>
+      <c r="G26">
+        <v>10</v>
+      </c>
+      <c r="H26">
+        <v>10</v>
+      </c>
+      <c r="I26">
+        <v>62</v>
+      </c>
+      <c r="J26">
+        <v>0.36299999999999999</v>
+      </c>
+      <c r="K26">
+        <v>0.46383333333333299</v>
+      </c>
+      <c r="L26" t="s">
+        <v>19</v>
+      </c>
+      <c r="M26" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>13</v>
+      </c>
+      <c r="B27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C27" t="s">
+        <v>28</v>
+      </c>
+      <c r="D27" t="s">
+        <v>16</v>
+      </c>
+      <c r="E27" t="s">
+        <v>17</v>
+      </c>
+      <c r="F27" t="s">
+        <v>21</v>
+      </c>
+      <c r="G27">
+        <v>10</v>
+      </c>
+      <c r="H27">
+        <v>10</v>
+      </c>
+      <c r="I27">
+        <v>43.5</v>
+      </c>
+      <c r="J27">
+        <v>0.63700000000000001</v>
+      </c>
+      <c r="K27">
+        <v>0.71917073170731705</v>
+      </c>
+      <c r="L27" t="s">
+        <v>19</v>
+      </c>
+      <c r="M27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>13</v>
+      </c>
+      <c r="B28" t="s">
+        <v>25</v>
+      </c>
+      <c r="C28" t="s">
+        <v>28</v>
+      </c>
+      <c r="D28" t="s">
+        <v>16</v>
+      </c>
+      <c r="E28" t="s">
+        <v>17</v>
+      </c>
+      <c r="F28" t="s">
+        <v>22</v>
+      </c>
+      <c r="G28">
+        <v>10</v>
+      </c>
+      <c r="H28">
+        <v>10</v>
+      </c>
+      <c r="I28">
+        <v>30</v>
+      </c>
+      <c r="J28">
+        <v>0.13100000000000001</v>
+      </c>
+      <c r="K28">
+        <v>0.20779310344827601</v>
+      </c>
+      <c r="L28" t="s">
+        <v>19</v>
+      </c>
+      <c r="M28" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>13</v>
+      </c>
+      <c r="B29" t="s">
+        <v>25</v>
+      </c>
+      <c r="C29" t="s">
+        <v>28</v>
+      </c>
+      <c r="D29" t="s">
+        <v>16</v>
+      </c>
+      <c r="E29" t="s">
+        <v>17</v>
+      </c>
+      <c r="F29" t="s">
+        <v>24</v>
+      </c>
+      <c r="G29">
+        <v>10</v>
+      </c>
+      <c r="H29">
+        <v>10</v>
+      </c>
+      <c r="I29">
+        <v>23.5</v>
+      </c>
+      <c r="J29">
+        <v>4.2000000000000003E-2</v>
+      </c>
+      <c r="K29">
+        <v>7.7280000000000001E-2</v>
+      </c>
+      <c r="L29" t="s">
+        <v>19</v>
+      </c>
+      <c r="M29" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>25</v>
+      </c>
+      <c r="C30" t="s">
+        <v>28</v>
+      </c>
+      <c r="D30" t="s">
+        <v>16</v>
+      </c>
+      <c r="E30" t="s">
+        <v>17</v>
+      </c>
+      <c r="F30" t="s">
+        <v>18</v>
+      </c>
+      <c r="G30">
+        <v>10</v>
+      </c>
+      <c r="H30">
+        <v>10</v>
+      </c>
+      <c r="I30">
         <v>0</v>
       </c>
-      <c r="J25" t="n">
-        <v>0.000145</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0.000602894736842105</v>
-      </c>
-      <c r="L25" t="s">
-        <v>23</v>
-      </c>
-      <c r="M25" t="s">
+      <c r="J30">
+        <v>1.44E-4</v>
+      </c>
+      <c r="K30">
+        <v>8.8933333333333301E-4</v>
+      </c>
+      <c r="L30" t="s">
+        <v>26</v>
+      </c>
+      <c r="M30" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" t="s">
+        <v>28</v>
+      </c>
+      <c r="D31" t="s">
+        <v>16</v>
+      </c>
+      <c r="E31" t="s">
+        <v>17</v>
+      </c>
+      <c r="F31" t="s">
+        <v>21</v>
+      </c>
+      <c r="G31">
+        <v>10</v>
+      </c>
+      <c r="H31">
+        <v>10</v>
+      </c>
+      <c r="I31">
+        <v>0</v>
+      </c>
+      <c r="J31">
+        <v>1.45E-4</v>
+      </c>
+      <c r="K31">
+        <v>8.8933333333333301E-4</v>
+      </c>
+      <c r="L31" t="s">
+        <v>26</v>
+      </c>
+      <c r="M31" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" t="s">
+        <v>25</v>
+      </c>
+      <c r="C32" t="s">
+        <v>28</v>
+      </c>
+      <c r="D32" t="s">
+        <v>16</v>
+      </c>
+      <c r="E32" t="s">
+        <v>17</v>
+      </c>
+      <c r="F32" t="s">
+        <v>22</v>
+      </c>
+      <c r="G32">
+        <v>10</v>
+      </c>
+      <c r="H32">
+        <v>10</v>
+      </c>
+      <c r="I32">
+        <v>0</v>
+      </c>
+      <c r="J32">
+        <v>1.44E-4</v>
+      </c>
+      <c r="K32">
+        <v>8.8933333333333301E-4</v>
+      </c>
+      <c r="L32" t="s">
+        <v>26</v>
+      </c>
+      <c r="M32" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>29</v>
+      </c>
+      <c r="B33" t="s">
+        <v>25</v>
+      </c>
+      <c r="C33" t="s">
+        <v>28</v>
+      </c>
+      <c r="D33" t="s">
+        <v>16</v>
+      </c>
+      <c r="E33" t="s">
+        <v>17</v>
+      </c>
+      <c r="F33" t="s">
+        <v>24</v>
+      </c>
+      <c r="G33">
+        <v>10</v>
+      </c>
+      <c r="H33">
+        <v>10</v>
+      </c>
+      <c r="I33">
+        <v>0</v>
+      </c>
+      <c r="J33">
+        <v>1.45E-4</v>
+      </c>
+      <c r="K33">
+        <v>8.8933333333333301E-4</v>
+      </c>
+      <c r="L33" t="s">
+        <v>26</v>
+      </c>
+      <c r="M33" t="s">
         <v>20</v>
       </c>
     </row>
   </sheetData>
+  <sortState ref="A2:M33">
+    <sortCondition ref="C1"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>